<commit_message>
fix: remove redundant Anticipo_Pct from legacy template, auto-populate amortized_advance from nc_advance_amount
</commit_message>
<xml_diff>
--- a/frontend/src/assets/plantilla-migracion-ov.xlsx
+++ b/frontend/src/assets/plantilla-migracion-ov.xlsx
@@ -456,20 +456,15 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Anticipo_Pct</t>
+          <t>Anticipo_Cobrado</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Anticipo_Cobrado</t>
+          <t>Comision_Pct</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
-        <is>
-          <t>Comision_Pct</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>

</xml_diff>

<commit_message>
feat: legacy import FG retention — optional due date column and real percent
- New optional Facturas column FG_Fecha_Vencimiento. When present it sets
  the retention due date (retention_days derived from invoice date). When
  missing and there is an FG credit note, due date = invoice date + OV
  retention days (90) with a visible warning showing the calculated date.
- Errors: due date without FG credit note, unreadable due date, due date
  before invoice date, NC_FG_Monto greater than Monto_Factura.
- retention_percent = NC_FG_Monto / Monto_Factura * 100 (4 decimals)
  instead of 0%, so imported retentions show in the order statement.
  retention_amount keeps the exact Excel amount.
- Template generator and downloadable template include the new column;
  regenerating also fixes OV example rows shifted by the old Anticipo_Pct.
  Generator logs instead of print().
- 12 new tests, including template/importer column parity.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/src/assets/plantilla-migracion-ov.xlsx
+++ b/frontend/src/assets/plantilla-migracion-ov.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,15 +493,12 @@
         <v>1160000</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>60</v>
+        <v>696000</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>696000</v>
-      </c>
-      <c r="H2" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="I2" s="1" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>Migración corte marzo 2026</t>
         </is>
@@ -530,15 +527,12 @@
         <v>580000</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>50</v>
+        <v>290000</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>290000</v>
-      </c>
-      <c r="H3" s="1" t="n">
         <v>2.5</v>
       </c>
-      <c r="I3" s="1" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>Solo saldos abiertos</t>
         </is>
@@ -555,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -606,30 +600,35 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>FG_Fecha_Vencimiento</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>Abono1_Fecha</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Abono1_Monto</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Abono2_Fecha</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Abono2_Monto</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Abono3_Fecha</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Abono3_Monto</t>
         </is>
@@ -667,20 +666,21 @@
       <c r="I2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="1" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr"/>
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>2025-11-20</t>
         </is>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="L2" s="1" t="n">
         <v>696000</v>
       </c>
-      <c r="L2" s="1" t="inlineStr"/>
-      <c r="M2" s="1" t="n">
+      <c r="M2" s="1" t="inlineStr"/>
+      <c r="N2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="1" t="inlineStr"/>
-      <c r="O2" s="1" t="n">
+      <c r="O2" s="1" t="inlineStr"/>
+      <c r="P2" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -720,24 +720,25 @@
       <c r="I3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="1" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr"/>
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>2026-01-15</t>
         </is>
       </c>
-      <c r="K3" s="1" t="n">
+      <c r="L3" s="1" t="n">
         <v>150000</v>
       </c>
-      <c r="L3" s="1" t="inlineStr">
+      <c r="M3" s="1" t="inlineStr">
         <is>
           <t>2026-02-01</t>
         </is>
       </c>
-      <c r="M3" s="1" t="n">
+      <c r="N3" s="1" t="n">
         <v>100000</v>
       </c>
-      <c r="N3" s="1" t="inlineStr"/>
-      <c r="O3" s="1" t="n">
+      <c r="O3" s="1" t="inlineStr"/>
+      <c r="P3" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -779,18 +780,23 @@
       </c>
       <c r="J4" s="1" t="inlineStr">
         <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
           <t>2025-12-05</t>
         </is>
       </c>
-      <c r="K4" s="1" t="n">
+      <c r="L4" s="1" t="n">
         <v>290000</v>
       </c>
-      <c r="L4" s="1" t="inlineStr"/>
-      <c r="M4" s="1" t="n">
+      <c r="M4" s="1" t="inlineStr"/>
+      <c r="N4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N4" s="1" t="inlineStr"/>
-      <c r="O4" s="1" t="n">
+      <c r="O4" s="1" t="inlineStr"/>
+      <c r="P4" s="1" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>